<commit_message>
feat(saisatwik): publish SAP PS spokes K12-K23, backdated 13-24 Oct
Twelve SAP PS cluster posts from the keyword workbook (K12-K23), live on
saisatwik.com as #5447-#5469, one per day from 13 Oct 2026.

- Runner: optional `date` in a data module is sent as WP date + date_gmt
  (site is UTC). Modules without it keep their existing WP date, so
  older posts and the hub are unaffected on re-run.
- Hub #5418 Related Reading now links down to all 12; forward links
  added between the new spokes after all were live.
- Workbook K12-K23 marked Published with live URLs; CLUSTERS.md and
  TAGS.md (new "Cheat Sheet" format tag) updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,8 +88,13 @@
       <b val="1"/>
       <color rgb="FF006100"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +128,11 @@
         <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -193,6 +203,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1339,9 +1350,14 @@
       <c r="H13" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I13" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-network-and-activities-explained/</t>
         </is>
       </c>
     </row>
@@ -1384,9 +1400,14 @@
       <c r="H14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-project-cost-planning-guide/</t>
         </is>
       </c>
     </row>
@@ -1429,9 +1450,14 @@
       <c r="H15" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I15" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J15" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/budgeting-and-availability-control-in-sap-ps/</t>
         </is>
       </c>
     </row>
@@ -1474,9 +1500,14 @@
       <c r="H16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/milestone-billing-in-sap-ps/</t>
         </is>
       </c>
     </row>
@@ -1519,9 +1550,14 @@
       <c r="H17" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I17" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J17" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/results-analysis-in-sap-ps-explained/</t>
         </is>
       </c>
     </row>
@@ -1564,9 +1600,14 @@
       <c r="H18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-settlement-explained/</t>
         </is>
       </c>
     </row>
@@ -1609,9 +1650,14 @@
       <c r="H19" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I19" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J19" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-and-fico-integration/</t>
         </is>
       </c>
     </row>
@@ -1654,9 +1700,14 @@
       <c r="H20" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I20" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J20" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-integration-with-mm-and-sd/</t>
         </is>
       </c>
     </row>
@@ -1699,9 +1750,14 @@
       <c r="H21" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I21" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J21" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/earned-value-management-in-sap-ps/</t>
         </is>
       </c>
     </row>
@@ -1744,9 +1800,14 @@
       <c r="H22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I22" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J22" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-transaction-codes-cheat-sheet/</t>
         </is>
       </c>
     </row>
@@ -1789,9 +1850,14 @@
       <c r="H23" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I23" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J23" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-in-s4hana-key-differences/</t>
         </is>
       </c>
     </row>
@@ -1834,9 +1900,14 @@
       <c r="H24" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I24" s="20" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J24" s="20" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-configuration-step-by-step/</t>
         </is>
       </c>
     </row>

</xml_diff>